<commit_message>
Pensumfiler Okonomistyring fra LOM_Pensum_2026_v2
</commit_message>
<xml_diff>
--- a/pensum/ok01/LOM_Ovingsark_Okonomistyring_kap01_Selskapsform_og_skatt_NY.xlsx
+++ b/pensum/ok01/LOM_Ovingsark_Okonomistyring_kap01_Selskapsform_og_skatt_NY.xlsx
@@ -790,7 +790,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>A3 · Klasseoppgave: Sara Lien vil starte for seg selv</t>
+          <t>A3 · Klasseoppgave: kan Sara starte for seg selv?</t>
         </is>
       </c>
       <c r="B30" s="8" t="inlineStr">
@@ -800,7 +800,7 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Legg Saras anslåtte tall i B5, B6 og B7, og les av D16 og D17.</t>
+          <t>Legg Saras anslåtte tall i B5, B6 og B7, og les av D16 og D17. Merk at arket bare svarer på det andre spørsmålet i oppgaven — det første, om hun kan tilby tjenesten, avgjøres av FEK § 7 og ikke av tall.</t>
         </is>
       </c>
     </row>
@@ -2563,6 +2563,13 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Forutsetning: han fyller selv FEK § 7 — fagskole, tre års praksis etter endt utdanning og installatørprøven — og kan stå som faglig ansvarlig. Uten det er selskapsform ikke hans første spørsmål.</t>
+        </is>
+      </c>
+    </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Versjon 2.2.0 · presentasjoner og pensum versjon 3
Alle 30 kapittelpresentasjoner byttet til versjon 3 (mer pensum, tydelige oppgaver, hovedpoeng). Sammendrag, hefter, regneark, faktaark og ordliste speilet fra LOM_Pensum_2026_v3 etter premisskontrollen.
</commit_message>
<xml_diff>
--- a/pensum/ok01/LOM_Ovingsark_Okonomistyring_kap01_Selskapsform_og_skatt_NY.xlsx
+++ b/pensum/ok01/LOM_Ovingsark_Okonomistyring_kap01_Selskapsform_og_skatt_NY.xlsx
@@ -608,6 +608,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -663,6 +664,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
@@ -691,6 +693,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
@@ -705,6 +708,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
@@ -729,6 +733,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
@@ -790,7 +795,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>A3 · Klasseoppgave: kan Sara starte for seg selv?</t>
+          <t>A3 · Klasseoppgave: kunne Tom startet alene?</t>
         </is>
       </c>
       <c r="B30" s="8" t="inlineStr">
@@ -800,7 +805,7 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Legg Saras anslåtte tall i B5, B6 og B7, og les av D16 og D17. Merk at arket bare svarer på det andre spørsmålet i oppgaven — det første, om hun kan tilby tjenesten, avgjøres av FEK § 7 og ikke av tall.</t>
+          <t>Legg anslåtte tall for første driftsår i B5, B6 og B7, og les av D16 og D17. Merk at arket bare svarer på det andre spørsmålet i oppgaven — det første, om foretaket kan tilby tjenesten, avgjøres av FEK § 7 og ikke av tall.</t>
         </is>
       </c>
     </row>
@@ -875,7 +880,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>5 · Eksamensnær: montøren som vil starte for seg selv</t>
+          <t>5 · Eksamensnær: installatøren som vil starte for seg selv</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
@@ -889,6 +894,7 @@
         </is>
       </c>
     </row>
+    <row r="36"/>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
@@ -917,6 +923,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
@@ -931,6 +938,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
@@ -1002,6 +1010,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -1080,6 +1089,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="9" t="inlineStr"/>
       <c r="B11" s="9" t="inlineStr">
@@ -1196,6 +1206,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
@@ -1280,6 +1291,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
@@ -1401,6 +1413,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
@@ -1441,6 +1454,7 @@
         <v/>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
@@ -1526,6 +1540,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -1593,6 +1608,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
@@ -1690,6 +1706,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
@@ -1745,6 +1762,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
@@ -1785,6 +1803,7 @@
         <v/>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
@@ -1851,6 +1870,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -1898,6 +1918,7 @@
         <v>18</v>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
@@ -2005,6 +2026,7 @@
         <v/>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
@@ -2061,6 +2083,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
@@ -2104,6 +2127,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
@@ -2133,6 +2157,7 @@
         <v/>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
@@ -2194,6 +2219,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -2208,6 +2234,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="9" t="inlineStr"/>
       <c r="B7" s="9" t="inlineStr">
@@ -2397,6 +2424,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
@@ -2415,6 +2443,8 @@
         <v/>
       </c>
     </row>
+    <row r="18"/>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
@@ -2429,6 +2459,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
@@ -2531,6 +2562,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
@@ -2549,10 +2581,12 @@
         <v/>
       </c>
     </row>
+    <row r="34"/>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Scenario C · montøren som vil starte for seg selv</t>
+          <t>Scenario C · installatøren som vil starte for seg selv</t>
         </is>
       </c>
     </row>
@@ -2647,6 +2681,7 @@
         <v/>
       </c>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
@@ -2752,6 +2787,7 @@
         </is>
       </c>
     </row>
+    <row r="55"/>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
@@ -2785,6 +2821,7 @@
         </is>
       </c>
     </row>
+    <row r="59"/>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
@@ -2832,6 +2869,7 @@
         <v/>
       </c>
     </row>
+    <row r="65"/>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>

</xml_diff>